<commit_message>
Excel actualizado ESPARTACO 2 con interpolación continuo grado 1
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -482,22 +482,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6562.318</v>
+        <v>6562.465</v>
       </c>
       <c r="D2" t="n">
-        <v>-7.499999999999999e-05</v>
+        <v>-5.3e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>-22.5534</v>
+        <v>-15.8409</v>
       </c>
       <c r="F2" t="n">
-        <v>0.34</v>
+        <v>0.3286</v>
       </c>
       <c r="G2" t="n">
-        <v>1.203</v>
+        <v>1.56</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5151</v>
+        <v>0.8719</v>
       </c>
     </row>
     <row r="3">
@@ -512,22 +512,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6562.961</v>
+        <v>6562.994</v>
       </c>
       <c r="D3" t="n">
-        <v>2.3e-05</v>
+        <v>2.8e-05</v>
       </c>
       <c r="E3" t="n">
-        <v>6.7908</v>
+        <v>8.301600000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7534999999999999</v>
+        <v>0.7981</v>
       </c>
       <c r="G3" t="n">
-        <v>1.153</v>
+        <v>1.051</v>
       </c>
       <c r="H3" t="n">
-        <v>1.1372</v>
+        <v>1.1102</v>
       </c>
     </row>
     <row r="4">
@@ -542,22 +542,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6563.901</v>
+        <v>6563.887</v>
       </c>
       <c r="D4" t="n">
-        <v>7.7e-05</v>
+        <v>7.499999999999999e-05</v>
       </c>
       <c r="E4" t="n">
-        <v>23</v>
+        <v>22.4002</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4094</v>
+        <v>0.4562</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.925</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4855</v>
+        <v>0.587</v>
       </c>
     </row>
     <row r="5">
@@ -572,22 +572,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6562.426</v>
+        <v>6562.499</v>
       </c>
       <c r="D5" t="n">
-        <v>-5.9e-05</v>
+        <v>-4.8e-05</v>
       </c>
       <c r="E5" t="n">
-        <v>-17.612</v>
+        <v>-14.3148</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3264</v>
+        <v>0.4783</v>
       </c>
       <c r="G5" t="n">
-        <v>1.263</v>
+        <v>1.233</v>
       </c>
       <c r="H5" t="n">
-        <v>0.453</v>
+        <v>0.9762</v>
       </c>
     </row>
     <row r="6">
@@ -602,22 +602,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6563.112</v>
+        <v>6563.101</v>
       </c>
       <c r="D6" t="n">
-        <v>4.6e-05</v>
+        <v>4.4e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>13.6934</v>
+        <v>13.1917</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8567</v>
+        <v>0.873</v>
       </c>
       <c r="G6" t="n">
-        <v>1.045</v>
+        <v>1.169</v>
       </c>
       <c r="H6" t="n">
-        <v>1.0711</v>
+        <v>1.1959</v>
       </c>
     </row>
     <row r="7">
@@ -641,13 +641,13 @@
         <v>28.7</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5532</v>
+        <v>0.5153</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.951</v>
       </c>
       <c r="H7" t="n">
-        <v>0.5725</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="8">
@@ -662,22 +662,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6562.135</v>
+        <v>6562.471</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.000103</v>
+        <v>-5.2e-05</v>
       </c>
       <c r="E8" t="n">
-        <v>-30.9362</v>
+        <v>-15.5775</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1727</v>
+        <v>0.3119</v>
       </c>
       <c r="G8" t="n">
-        <v>1.027</v>
+        <v>1.588</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2117</v>
+        <v>0.8761</v>
       </c>
     </row>
     <row r="9">
@@ -692,22 +692,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6563.191</v>
+        <v>6563.166</v>
       </c>
       <c r="D9" t="n">
-        <v>5.8e-05</v>
+        <v>5.4e-05</v>
       </c>
       <c r="E9" t="n">
-        <v>17.3336</v>
+        <v>16.1646</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6312</v>
+        <v>0.7344000000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9370000000000001</v>
+        <v>1.118</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7060999999999999</v>
+        <v>1.0396</v>
       </c>
     </row>
     <row r="10">
@@ -731,13 +731,13 @@
         <v>29.3</v>
       </c>
       <c r="F10" t="n">
-        <v>0.556</v>
+        <v>0.4768</v>
       </c>
       <c r="G10" t="n">
-        <v>0.971</v>
+        <v>0.987</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6551</v>
+        <v>0.6306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adición de estimación del continuo
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Julio-2026</t>
+          <t>Septiembre 06-2025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,28 +482,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6562.465</v>
+        <v>6562.467</v>
       </c>
       <c r="D2" t="n">
         <v>-5.3e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>-15.8409</v>
+        <v>-15.7495</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3286</v>
+        <v>0.3103</v>
       </c>
       <c r="G2" t="n">
-        <v>1.56</v>
+        <v>1.586</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8719</v>
+        <v>0.8702</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Julio-2026</t>
+          <t>Septiembre 06-2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -512,28 +512,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6562.994</v>
+        <v>6563.166</v>
       </c>
       <c r="D3" t="n">
-        <v>2.8e-05</v>
+        <v>5.4e-05</v>
       </c>
       <c r="E3" t="n">
-        <v>8.301600000000001</v>
+        <v>16.19</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7981</v>
+        <v>0.7326</v>
       </c>
       <c r="G3" t="n">
-        <v>1.051</v>
+        <v>1.117</v>
       </c>
       <c r="H3" t="n">
-        <v>1.1102</v>
+        <v>1.0358</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Julio-2026</t>
+          <t>Septiembre 06-2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -542,28 +542,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6563.887</v>
+        <v>6564.038</v>
       </c>
       <c r="D4" t="n">
-        <v>7.499999999999999e-05</v>
+        <v>9.8e-05</v>
       </c>
       <c r="E4" t="n">
-        <v>22.4002</v>
+        <v>29.3</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4562</v>
+        <v>0.4768</v>
       </c>
       <c r="G4" t="n">
-        <v>0.925</v>
+        <v>0.986</v>
       </c>
       <c r="H4" t="n">
-        <v>0.587</v>
+        <v>0.6302</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Agosto-2026</t>
+          <t>Julio 22-2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -572,28 +572,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6562.499</v>
+        <v>6562.445</v>
       </c>
       <c r="D5" t="n">
-        <v>-4.8e-05</v>
+        <v>-5.6e-05</v>
       </c>
       <c r="E5" t="n">
-        <v>-14.3148</v>
+        <v>-16.7831</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4783</v>
+        <v>0.3252</v>
       </c>
       <c r="G5" t="n">
-        <v>1.233</v>
+        <v>1.531</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9762</v>
+        <v>0.8512999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Agosto-2026</t>
+          <t>Julio 22-2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -602,28 +602,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6563.101</v>
+        <v>6562.991</v>
       </c>
       <c r="D6" t="n">
-        <v>4.4e-05</v>
+        <v>2.7e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>13.1917</v>
+        <v>8.184799999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.873</v>
+        <v>0.7864</v>
       </c>
       <c r="G6" t="n">
-        <v>1.169</v>
+        <v>1.051</v>
       </c>
       <c r="H6" t="n">
-        <v>1.1959</v>
+        <v>1.0932</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Agosto-2026</t>
+          <t>Julio 22-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -632,28 +632,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6564.025</v>
+        <v>6563.885</v>
       </c>
       <c r="D7" t="n">
-        <v>9.6e-05</v>
+        <v>7.4e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>28.7</v>
+        <v>22.277</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5153</v>
+        <v>0.4563</v>
       </c>
       <c r="G7" t="n">
-        <v>0.951</v>
+        <v>0.925</v>
       </c>
       <c r="H7" t="n">
-        <v>0.609</v>
+        <v>0.587</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Septiembre-2025</t>
+          <t>Julio 24-2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -662,28 +662,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6562.471</v>
+        <v>6562.045</v>
       </c>
       <c r="D8" t="n">
-        <v>-5.2e-05</v>
+        <v>-0.000117</v>
       </c>
       <c r="E8" t="n">
-        <v>-15.5775</v>
+        <v>-35.0176</v>
       </c>
       <c r="F8" t="n">
-        <v>0.3119</v>
+        <v>0.2894</v>
       </c>
       <c r="G8" t="n">
-        <v>1.588</v>
+        <v>1.098</v>
       </c>
       <c r="H8" t="n">
-        <v>0.8761</v>
+        <v>0.4706</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Septiembre-2025</t>
+          <t>Julio 24-2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -692,28 +692,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6563.166</v>
+        <v>6562.838</v>
       </c>
       <c r="D9" t="n">
-        <v>5.4e-05</v>
+        <v>4e-06</v>
       </c>
       <c r="E9" t="n">
-        <v>16.1646</v>
+        <v>1.2047</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7344000000000001</v>
+        <v>0.6938</v>
       </c>
       <c r="G9" t="n">
-        <v>1.118</v>
+        <v>1.233</v>
       </c>
       <c r="H9" t="n">
-        <v>1.0396</v>
+        <v>1.0572</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Septiembre-2025</t>
+          <t>Julio 24-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -722,22 +722,652 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6564.038</v>
+        <v>6563.793</v>
       </c>
       <c r="D10" t="n">
-        <v>9.8e-05</v>
+        <v>6e-05</v>
       </c>
       <c r="E10" t="n">
-        <v>29.3</v>
+        <v>18.07</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4768</v>
+        <v>0.4883</v>
       </c>
       <c r="G10" t="n">
-        <v>0.987</v>
+        <v>1.027</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6306</v>
+        <v>0.6548</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6561.895</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.00014</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-41.9106</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.2092</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.2427</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6562.888</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.2e-05</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.4787</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.6595</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.9411</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6563.795</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6.1e-05</v>
+      </c>
+      <c r="E13" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.5003</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.6554</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6562.122</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.000105</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-31.521</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.3159</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.031</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.397</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6562.868</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9e-06</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.5632</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.6921</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.269</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.0701</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6563.849</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6.9e-05</v>
+      </c>
+      <c r="E16" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.4954</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.6525</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6562.174</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-9.7e-05</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-29.1421</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.3824</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.5965</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6562.876</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.9311</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.7339</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.304</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1.1608</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>6563.874</v>
+      </c>
+      <c r="D19" t="n">
+        <v>7.3e-05</v>
+      </c>
+      <c r="E19" t="n">
+        <v>21.7699</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.4977</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.041</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.6685</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>6562.168</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-9.8e-05</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-29.4391</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.3499</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.112</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.5459000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6562.873</v>
+      </c>
+      <c r="D21" t="n">
+        <v>9e-06</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.8079</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.7166</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.313</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1.1551</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6563.87</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7.2e-05</v>
+      </c>
+      <c r="E22" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.4917</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6562.48</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-5.1e-05</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-15.1797</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.4423</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1.244</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.9103</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>6563.114</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4.6e-05</v>
+      </c>
+      <c r="E24" t="n">
+        <v>13.8034</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.8505</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1.145</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>6564.025</v>
+      </c>
+      <c r="D25" t="n">
+        <v>9.6e-05</v>
+      </c>
+      <c r="E25" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.5155999999999999</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.6068</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>6562.139</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.000102</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-30.7243</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.3018</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.4681</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>6562.98</v>
+      </c>
+      <c r="D27" t="n">
+        <v>2.6e-05</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7.6944</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.7611</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1.281</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.0762</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>6563.948</v>
+      </c>
+      <c r="D28" t="n">
+        <v>8.4e-05</v>
+      </c>
+      <c r="E28" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.5489000000000001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.698</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Septiembre 07-2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6562.106</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-0.000108</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-32.2412</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.2978</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.4256</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Septiembre 07-2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>6562.949</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2.1e-05</v>
+      </c>
+      <c r="E30" t="n">
+        <v>6.246</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.7348</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1.307</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1.0735</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Septiembre 07-2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>6563.924</v>
+      </c>
+      <c r="D31" t="n">
+        <v>8.000000000000001e-05</v>
+      </c>
+      <c r="E31" t="n">
+        <v>24.07</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.5484</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1.126</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.7531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perfil cada 4 filas
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/resultados perfiles halpha 2025 y 2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Septiembre 06-2025</t>
+          <t>Julio 11-2024</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,28 +482,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6562.467</v>
+        <v>6562.448</v>
       </c>
       <c r="D2" t="n">
-        <v>-5.3e-05</v>
+        <v>-5.5e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>-15.7495</v>
+        <v>-16.6369</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3103</v>
+        <v>0.3898</v>
       </c>
       <c r="G2" t="n">
-        <v>1.586</v>
+        <v>1.555</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8702</v>
+        <v>0.9323</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Septiembre 06-2025</t>
+          <t>Julio 11-2024</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -512,28 +512,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6563.166</v>
+        <v>6562.905</v>
       </c>
       <c r="D3" t="n">
-        <v>5.4e-05</v>
+        <v>1.4e-05</v>
       </c>
       <c r="E3" t="n">
-        <v>16.19</v>
+        <v>4.2427</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7326</v>
+        <v>0.9122</v>
       </c>
       <c r="G3" t="n">
-        <v>1.117</v>
+        <v>1.059</v>
       </c>
       <c r="H3" t="n">
-        <v>1.0358</v>
+        <v>1.1795</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Septiembre 06-2025</t>
+          <t>Julio 11-2024</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -542,28 +542,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6564.038</v>
+        <v>6563.815</v>
       </c>
       <c r="D4" t="n">
-        <v>9.8e-05</v>
+        <v>6.4e-05</v>
       </c>
       <c r="E4" t="n">
-        <v>29.3</v>
+        <v>19.0999</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4768</v>
+        <v>0.4944</v>
       </c>
       <c r="G4" t="n">
-        <v>0.986</v>
+        <v>0.927</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6302</v>
+        <v>0.5872000000000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Julio 22-2026</t>
+          <t>Julio 22-2024</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -572,28 +572,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6562.47</v>
+        <v>6561.996</v>
       </c>
       <c r="D5" t="n">
-        <v>-5.2e-05</v>
+        <v>-0.000124</v>
       </c>
       <c r="E5" t="n">
-        <v>-15.6295</v>
+        <v>-37.2771</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3294</v>
+        <v>0.1879</v>
       </c>
       <c r="G5" t="n">
-        <v>1.567</v>
+        <v>0.982</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8764999999999999</v>
+        <v>0.2444</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Julio 22-2026</t>
+          <t>Julio 22-2024</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -602,28 +602,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6562.994</v>
+        <v>6563.038</v>
       </c>
       <c r="D6" t="n">
-        <v>2.8e-05</v>
+        <v>3.4e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>8.3309</v>
+        <v>10.3394</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8007</v>
+        <v>0.6215000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>1.051</v>
+        <v>0.875</v>
       </c>
       <c r="H6" t="n">
-        <v>1.114</v>
+        <v>0.6232</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Julio 22-2026</t>
+          <t>Julio 22-2024</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -632,28 +632,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6563.888</v>
+        <v>6563.876</v>
       </c>
       <c r="D7" t="n">
-        <v>7.499999999999999e-05</v>
+        <v>7.3e-05</v>
       </c>
       <c r="E7" t="n">
-        <v>22.4289</v>
+        <v>21.86</v>
       </c>
       <c r="F7" t="n">
-        <v>0.4562</v>
+        <v>0.5265</v>
       </c>
       <c r="G7" t="n">
-        <v>0.925</v>
+        <v>0.883</v>
       </c>
       <c r="H7" t="n">
-        <v>0.587</v>
+        <v>0.5611</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Julio 24-2026</t>
+          <t>Agosto 16-2024</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -662,28 +662,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6562.042</v>
+        <v>6562.542</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.000117</v>
+        <v>-4.1e-05</v>
       </c>
       <c r="E8" t="n">
-        <v>-35.1772</v>
+        <v>-12.3499</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2865</v>
+        <v>0.5289</v>
       </c>
       <c r="G8" t="n">
-        <v>1.096</v>
+        <v>1.223</v>
       </c>
       <c r="H8" t="n">
-        <v>0.4654</v>
+        <v>0.9347</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Julio 24-2026</t>
+          <t>Agosto 16-2024</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -692,28 +692,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6562.84</v>
+        <v>6563.025</v>
       </c>
       <c r="D9" t="n">
-        <v>4e-06</v>
+        <v>3.2e-05</v>
       </c>
       <c r="E9" t="n">
-        <v>1.2967</v>
+        <v>9.7233</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6921</v>
+        <v>0.9089</v>
       </c>
       <c r="G9" t="n">
-        <v>1.23</v>
+        <v>1.164</v>
       </c>
       <c r="H9" t="n">
-        <v>1.0524</v>
+        <v>1.309</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Julio 24-2026</t>
+          <t>Agosto 16-2024</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -722,28 +722,28 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6563.793</v>
+        <v>6563.998</v>
       </c>
       <c r="D10" t="n">
-        <v>6e-05</v>
+        <v>9.2e-05</v>
       </c>
       <c r="E10" t="n">
-        <v>18.07</v>
+        <v>27.47</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4883</v>
+        <v>0.4879</v>
       </c>
       <c r="G10" t="n">
-        <v>1.027</v>
+        <v>0.926</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6546999999999999</v>
+        <v>0.5868</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Julio 27-2026</t>
+          <t>Agosto 26-2024</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -752,28 +752,28 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6561.91</v>
+        <v>6562.498</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.000138</v>
+        <v>-4.8e-05</v>
       </c>
       <c r="E11" t="n">
-        <v>-41.2233</v>
+        <v>-14.3455</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2118</v>
+        <v>0.5451</v>
       </c>
       <c r="G11" t="n">
-        <v>0.968</v>
+        <v>1.117</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2474</v>
+        <v>0.8788</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Julio 27-2026</t>
+          <t>Agosto 26-2024</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -782,28 +782,28 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6562.883</v>
+        <v>6563.045</v>
       </c>
       <c r="D12" t="n">
-        <v>1.1e-05</v>
+        <v>3.5e-05</v>
       </c>
       <c r="E12" t="n">
-        <v>3.2596</v>
+        <v>10.6416</v>
       </c>
       <c r="F12" t="n">
-        <v>0.656</v>
+        <v>0.9061</v>
       </c>
       <c r="G12" t="n">
-        <v>1.143</v>
+        <v>1.208</v>
       </c>
       <c r="H12" t="n">
-        <v>0.9317</v>
+        <v>1.2492</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Julio 27-2026</t>
+          <t>Agosto 26-2024</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -812,28 +812,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6563.795</v>
+        <v>6564.025</v>
       </c>
       <c r="D13" t="n">
-        <v>6.1e-05</v>
+        <v>9.6e-05</v>
       </c>
       <c r="E13" t="n">
-        <v>18.19</v>
+        <v>28.69</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5003</v>
+        <v>0.5288</v>
       </c>
       <c r="G13" t="n">
-        <v>1.041</v>
+        <v>0.968</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6685</v>
+        <v>0.6183</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Agosto 06-2026</t>
+          <t>Septiembre 06-2024</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -842,28 +842,28 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6562.122</v>
+        <v>6562.495</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.000105</v>
+        <v>-4.8e-05</v>
       </c>
       <c r="E14" t="n">
-        <v>-31.521</v>
+        <v>-14.4749</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3159</v>
+        <v>0.3796</v>
       </c>
       <c r="G14" t="n">
-        <v>1.031</v>
+        <v>1.317</v>
       </c>
       <c r="H14" t="n">
-        <v>0.397</v>
+        <v>0.8424</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Agosto 06-2026</t>
+          <t>Septiembre 06-2024</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -872,28 +872,28 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>6562.868</v>
+        <v>6563.104</v>
       </c>
       <c r="D15" t="n">
-        <v>9e-06</v>
+        <v>4.5e-05</v>
       </c>
       <c r="E15" t="n">
-        <v>2.5632</v>
+        <v>13.357</v>
       </c>
       <c r="F15" t="n">
-        <v>0.6921</v>
+        <v>0.7659</v>
       </c>
       <c r="G15" t="n">
-        <v>1.269</v>
+        <v>1.175</v>
       </c>
       <c r="H15" t="n">
-        <v>1.0701</v>
+        <v>1.1158</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Agosto 06-2026</t>
+          <t>Septiembre 06-2024</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -902,28 +902,28 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6563.849</v>
+        <v>6564.027</v>
       </c>
       <c r="D16" t="n">
-        <v>6.9e-05</v>
+        <v>9.6e-05</v>
       </c>
       <c r="E16" t="n">
-        <v>20.64</v>
+        <v>28.76</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4954</v>
+        <v>0.4869</v>
       </c>
       <c r="G16" t="n">
-        <v>1.025</v>
+        <v>1.008</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6525</v>
+        <v>0.6425999999999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Agosto 10-2026</t>
+          <t>Septiembre 19-2024</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -932,28 +932,28 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>6562.174</v>
+        <v>6562.365</v>
       </c>
       <c r="D17" t="n">
-        <v>-9.7e-05</v>
+        <v>-6.8e-05</v>
       </c>
       <c r="E17" t="n">
-        <v>-29.1421</v>
+        <v>-20.4338</v>
       </c>
       <c r="F17" t="n">
-        <v>0.3824</v>
+        <v>0.2681</v>
       </c>
       <c r="G17" t="n">
-        <v>1.133</v>
+        <v>1.281</v>
       </c>
       <c r="H17" t="n">
-        <v>0.5965</v>
+        <v>0.4125</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Agosto 10-2026</t>
+          <t>Septiembre 19-2024</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -962,28 +962,28 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6562.876</v>
+        <v>6563.101</v>
       </c>
       <c r="D18" t="n">
-        <v>1e-05</v>
+        <v>4.4e-05</v>
       </c>
       <c r="E18" t="n">
-        <v>2.9311</v>
+        <v>13.2045</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7339</v>
+        <v>0.6959</v>
       </c>
       <c r="G18" t="n">
-        <v>1.304</v>
+        <v>1.095</v>
       </c>
       <c r="H18" t="n">
-        <v>1.1608</v>
+        <v>0.915</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Agosto 10-2026</t>
+          <t>Septiembre 19-2024</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -992,28 +992,28 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>6563.874</v>
+        <v>6564.004</v>
       </c>
       <c r="D19" t="n">
-        <v>7.3e-05</v>
+        <v>9.2e-05</v>
       </c>
       <c r="E19" t="n">
-        <v>21.7699</v>
+        <v>27.73</v>
       </c>
       <c r="F19" t="n">
-        <v>0.4977</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>1.041</v>
+        <v>1.002</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6685</v>
+        <v>0.639</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Agosto 13-2026</t>
+          <t>Septiembre 24-2024</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1022,28 +1022,28 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6562.168</v>
+        <v>6562.444</v>
       </c>
       <c r="D20" t="n">
-        <v>-9.8e-05</v>
+        <v>-5.6e-05</v>
       </c>
       <c r="E20" t="n">
-        <v>-29.4391</v>
+        <v>-16.8025</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3499</v>
+        <v>0.4913</v>
       </c>
       <c r="G20" t="n">
-        <v>1.112</v>
+        <v>1.14</v>
       </c>
       <c r="H20" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.7803</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Agosto 13-2026</t>
+          <t>Septiembre 24-2024</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1052,28 +1052,28 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6562.873</v>
+        <v>6562.999</v>
       </c>
       <c r="D21" t="n">
-        <v>9e-06</v>
+        <v>2.8e-05</v>
       </c>
       <c r="E21" t="n">
-        <v>2.8079</v>
+        <v>8.5372</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7166</v>
+        <v>0.7731</v>
       </c>
       <c r="G21" t="n">
-        <v>1.313</v>
+        <v>1.268</v>
       </c>
       <c r="H21" t="n">
-        <v>1.1551</v>
+        <v>1.1841</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Agosto 13-2026</t>
+          <t>Septiembre 24-2024</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1082,28 +1082,28 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6563.87</v>
+        <v>6563.991</v>
       </c>
       <c r="D22" t="n">
-        <v>7.2e-05</v>
+        <v>9.1e-05</v>
       </c>
       <c r="E22" t="n">
-        <v>21.59</v>
+        <v>27.14</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4917</v>
+        <v>0.4998</v>
       </c>
       <c r="G22" t="n">
-        <v>1.052</v>
+        <v>1.041</v>
       </c>
       <c r="H22" t="n">
-        <v>0.68</v>
+        <v>0.6685</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Agosto 26-2026</t>
+          <t>Octubre 01-2024</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1112,28 +1112,28 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6562.48</v>
+        <v>6562.389</v>
       </c>
       <c r="D23" t="n">
-        <v>-5.1e-05</v>
+        <v>-6.499999999999999e-05</v>
       </c>
       <c r="E23" t="n">
-        <v>-15.1797</v>
+        <v>-19.3429</v>
       </c>
       <c r="F23" t="n">
-        <v>0.4423</v>
+        <v>0.4258</v>
       </c>
       <c r="G23" t="n">
-        <v>1.244</v>
+        <v>1.119</v>
       </c>
       <c r="H23" t="n">
-        <v>0.9103</v>
+        <v>0.5682</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Agosto 26-2026</t>
+          <t>Octubre 01-2024</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1142,28 +1142,28 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6563.114</v>
+        <v>6563.008</v>
       </c>
       <c r="D24" t="n">
-        <v>4.6e-05</v>
+        <v>3e-05</v>
       </c>
       <c r="E24" t="n">
-        <v>13.8034</v>
+        <v>8.9337</v>
       </c>
       <c r="F24" t="n">
-        <v>0.8505</v>
+        <v>0.7266</v>
       </c>
       <c r="G24" t="n">
-        <v>1.15</v>
+        <v>1.234</v>
       </c>
       <c r="H24" t="n">
-        <v>1.145</v>
+        <v>1.069</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Agosto 26-2026</t>
+          <t>Octubre 01-2024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1172,28 +1172,28 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>6564.025</v>
+        <v>6563.982</v>
       </c>
       <c r="D25" t="n">
-        <v>9.6e-05</v>
+        <v>8.899999999999999e-05</v>
       </c>
       <c r="E25" t="n">
-        <v>28.7</v>
+        <v>26.71</v>
       </c>
       <c r="F25" t="n">
-        <v>0.5155999999999999</v>
+        <v>0.5061</v>
       </c>
       <c r="G25" t="n">
-        <v>0.947</v>
+        <v>1.025</v>
       </c>
       <c r="H25" t="n">
-        <v>0.6068</v>
+        <v>0.6525</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Agosto 28-2026</t>
+          <t>Octubre 11-2024</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1202,28 +1202,28 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6562.139</v>
+        <v>6562.299</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.000102</v>
+        <v>-7.8e-05</v>
       </c>
       <c r="E26" t="n">
-        <v>-30.7243</v>
+        <v>-23.4498</v>
       </c>
       <c r="F26" t="n">
-        <v>0.3018</v>
+        <v>0.4244</v>
       </c>
       <c r="G26" t="n">
-        <v>1.095</v>
+        <v>1.264</v>
       </c>
       <c r="H26" t="n">
-        <v>0.4681</v>
+        <v>0.7702</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Agosto 28-2026</t>
+          <t>Octubre 11-2024</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1232,28 +1232,28 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6562.98</v>
+        <v>6562.986</v>
       </c>
       <c r="D27" t="n">
         <v>2.6e-05</v>
       </c>
       <c r="E27" t="n">
-        <v>7.6944</v>
+        <v>7.9443</v>
       </c>
       <c r="F27" t="n">
-        <v>0.7611</v>
+        <v>0.825</v>
       </c>
       <c r="G27" t="n">
-        <v>1.281</v>
+        <v>1.177</v>
       </c>
       <c r="H27" t="n">
-        <v>1.0762</v>
+        <v>1.2804</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Agosto 28-2026</t>
+          <t>Octubre 11-2024</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1262,28 +1262,28 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6563.948</v>
+        <v>6563.893</v>
       </c>
       <c r="D28" t="n">
-        <v>8.4e-05</v>
+        <v>7.6e-05</v>
       </c>
       <c r="E28" t="n">
-        <v>25.15</v>
+        <v>22.64</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.5544</v>
       </c>
       <c r="G28" t="n">
-        <v>1.07</v>
+        <v>1.053</v>
       </c>
       <c r="H28" t="n">
-        <v>0.698</v>
+        <v>0.6811</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Septiembre 07-2026</t>
+          <t>Octubre 17-2024</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1292,28 +1292,28 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6562.106</v>
+        <v>6562.212</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.000108</v>
+        <v>-9.1e-05</v>
       </c>
       <c r="E29" t="n">
-        <v>-32.2412</v>
+        <v>-27.4297</v>
       </c>
       <c r="F29" t="n">
-        <v>0.2978</v>
+        <v>0.3821</v>
       </c>
       <c r="G29" t="n">
-        <v>1.046</v>
+        <v>1.244</v>
       </c>
       <c r="H29" t="n">
-        <v>0.4256</v>
+        <v>0.6911</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Septiembre 07-2026</t>
+          <t>Octubre 17-2024</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1322,51 +1322,1131 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6562.949</v>
+        <v>6562.939</v>
       </c>
       <c r="D30" t="n">
-        <v>2.1e-05</v>
+        <v>1.9e-05</v>
       </c>
       <c r="E30" t="n">
-        <v>6.246</v>
+        <v>5.8222</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7348</v>
+        <v>0.7957</v>
       </c>
       <c r="G30" t="n">
-        <v>1.307</v>
+        <v>1.154</v>
       </c>
       <c r="H30" t="n">
-        <v>1.0735</v>
+        <v>1.1765</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Octubre 17-2024</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>6563.84</v>
+      </c>
+      <c r="D31" t="n">
+        <v>6.8e-05</v>
+      </c>
+      <c r="E31" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.5538</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1.043</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.6707</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Octubre 18-2024</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>6562.21</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-9.2e-05</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-27.5046</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3988</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1.093</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.5226</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Octubre 18-2024</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>6562.873</v>
+      </c>
+      <c r="D33" t="n">
+        <v>9e-06</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.7643</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.6762</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1.252</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1.0153</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Octubre 18-2024</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>6563.83</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6.600000000000001e-05</v>
+      </c>
+      <c r="E34" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.5034999999999999</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.6525</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Octubre 24-2024</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>6562.111</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-0.000107</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-32.0071</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.3881</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.4802</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Octubre 24-2024</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>6562.878</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3.0169</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1.231</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1.0231</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Octubre 24-2024</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>6563.788</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6e-05</v>
+      </c>
+      <c r="E37" t="n">
+        <v>17.87</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.5184</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.6683</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Septiembre 06-2025</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>6562.463</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-5.3e-05</v>
+      </c>
+      <c r="E38" t="n">
+        <v>-15.9468</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.3083</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1.583</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.8633</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Septiembre 06-2025</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6563.167</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5.4e-05</v>
+      </c>
+      <c r="E39" t="n">
+        <v>16.2206</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.7306</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1.115</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1.0315</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Septiembre 06-2025</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6564.038</v>
+      </c>
+      <c r="D40" t="n">
+        <v>9.8e-05</v>
+      </c>
+      <c r="E40" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.4769</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.6297</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Julio 22-2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>6562.406</v>
+      </c>
+      <c r="D41" t="n">
+        <v>-6.2e-05</v>
+      </c>
+      <c r="E41" t="n">
+        <v>-18.5634</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.3182</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1.476</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.8136</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Julio 22-2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>6562.988</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2.7e-05</v>
+      </c>
+      <c r="E42" t="n">
+        <v>8.037800000000001</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.7635</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.0606</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Julio 22-2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>6563.88</v>
+      </c>
+      <c r="D43" t="n">
+        <v>7.4e-05</v>
+      </c>
+      <c r="E43" t="n">
+        <v>22.069</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.587</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Julio 24-2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>6562.019</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-0.000121</v>
+      </c>
+      <c r="E44" t="n">
+        <v>-36.2429</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.4337</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Julio 24-2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>6562.853</v>
+      </c>
+      <c r="D45" t="n">
+        <v>6e-06</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.8737</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.6818</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.214</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.0234</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Julio 24-2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>6563.793</v>
+      </c>
+      <c r="D46" t="n">
+        <v>6e-05</v>
+      </c>
+      <c r="E46" t="n">
+        <v>18.07</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.4884</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.6531</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>6561.891</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-0.00014</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-42.063</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.2086</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.2413</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>6562.889</v>
+      </c>
+      <c r="D48" t="n">
+        <v>1.2e-05</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3.5257</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.6597</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.9416</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Julio 27-2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>6563.795</v>
+      </c>
+      <c r="D49" t="n">
+        <v>6.1e-05</v>
+      </c>
+      <c r="E49" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.5004</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.6543</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>6562.148</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-0.000101</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-30.3483</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.3547</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1.051</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.4543</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>6562.842</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5e-06</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1.3536</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.716</v>
+      </c>
+      <c r="G51" t="n">
+        <v>1.293</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1.128</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Agosto 06-2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6563.849</v>
+      </c>
+      <c r="D52" t="n">
+        <v>6.9e-05</v>
+      </c>
+      <c r="E52" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.4954</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.6525</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>6562.177</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-9.7e-05</v>
+      </c>
+      <c r="E53" t="n">
+        <v>-29.0068</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.3875</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.6049</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>6562.873</v>
+      </c>
+      <c r="D54" t="n">
+        <v>9e-06</v>
+      </c>
+      <c r="E54" t="n">
+        <v>2.7949</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.7371</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1.307</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1.1687</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Agosto 10-2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>6563.874</v>
+      </c>
+      <c r="D55" t="n">
+        <v>7.3e-05</v>
+      </c>
+      <c r="E55" t="n">
+        <v>21.77</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.4977</v>
+      </c>
+      <c r="G55" t="n">
+        <v>1.041</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.6685</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>6562.166</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-9.8e-05</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-29.5136</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.3471</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1.111</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.5417</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>6562.875</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1e-05</v>
+      </c>
+      <c r="E57" t="n">
+        <v>2.8908</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.7149</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1.311</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1.1508</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Agosto 13-2026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>6563.87</v>
+      </c>
+      <c r="D58" t="n">
+        <v>7.2e-05</v>
+      </c>
+      <c r="E58" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.4917</v>
+      </c>
+      <c r="G58" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.6801</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>6562.486</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-5e-05</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-14.8782</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.4537</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1.241</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.9314</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>6563.11</v>
+      </c>
+      <c r="D60" t="n">
+        <v>4.5e-05</v>
+      </c>
+      <c r="E60" t="n">
+        <v>13.6078</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.8577</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1.156</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1.1613</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Agosto 26-2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>6564.025</v>
+      </c>
+      <c r="D61" t="n">
+        <v>9.6e-05</v>
+      </c>
+      <c r="E61" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.5155</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.6075</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>6562.141</v>
+      </c>
+      <c r="D62" t="n">
+        <v>-0.000102</v>
+      </c>
+      <c r="E62" t="n">
+        <v>-30.6728</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.3028</v>
+      </c>
+      <c r="G62" t="n">
+        <v>1.096</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.469</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>6562.98</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2.6e-05</v>
+      </c>
+      <c r="E63" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.7614</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1.282</v>
+      </c>
+      <c r="H63" t="n">
+        <v>1.077</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Agosto 28-2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Absorción Cobalto</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>6563.948</v>
+      </c>
+      <c r="D64" t="n">
+        <v>8.4e-05</v>
+      </c>
+      <c r="E64" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.5489000000000001</v>
+      </c>
+      <c r="G64" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.6982</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>Septiembre 07-2026</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Emisión Azul Hα</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>6562.106</v>
+      </c>
+      <c r="D65" t="n">
+        <v>-0.000108</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-32.2395</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.2979</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1.046</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.4257</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Septiembre 07-2026</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Absorción Hα</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>6562.949</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2.1e-05</v>
+      </c>
+      <c r="E66" t="n">
+        <v>6.2449</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.7348</v>
+      </c>
+      <c r="G66" t="n">
+        <v>1.307</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1.0736</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Septiembre 07-2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>Absorción Cobalto</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C67" t="n">
         <v>6563.924</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D67" t="n">
         <v>8.000000000000001e-05</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E67" t="n">
         <v>24.07</v>
       </c>
-      <c r="F31" t="n">
+      <c r="F67" t="n">
         <v>0.5484</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G67" t="n">
         <v>1.126</v>
       </c>
-      <c r="H31" t="n">
+      <c r="H67" t="n">
         <v>0.7531</v>
       </c>
     </row>

</xml_diff>